<commit_message>
refactor: move get_code_map.py, update paths and fix typos in 12-upload_file_merge_file/
</commit_message>
<xml_diff>
--- a/12-upload_file_merge_file/output/pub_cd_map.xlsx
+++ b/12-upload_file_merge_file/output/pub_cd_map.xlsx
@@ -1,39 +1,192 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\12-upload_file_merge_file\output\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87441041-F18D-4D5F-8A53-F8EAAF4E43FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="23452" windowHeight="12561" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="rem-代码映射" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+  <si>
+    <t>取数来源应用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>取数来源表中文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>取数来源表英文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>取数来源字段中文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>取数来源字段英文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>源代码码值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>源代码码值说明</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标表中文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标表英文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标字段中文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标字段英文名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标代码码值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标代码说明</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>特殊说明</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>REM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGET_CD_DESC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGET_CD_VAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGRT_FIELD_CN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGRT_FIELD_EN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGRT_TAB_CN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TARGRT_TAB_EN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_CD_DESC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_CD_VAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_FIELD_CN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_FIELD_EN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_TAB_CN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_TAB_EN_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SRC_TAB_LIB_NAME</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>line4444444</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -41,85 +194,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -385,14 +498,194 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultRowHeight="13.95" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="4" max="14" width="14.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="22.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>111</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+      <c r="N3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>111</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance code mapping and progress tracking in app.py
</commit_message>
<xml_diff>
--- a/12-upload_file_merge_file/output/pub_cd_map.xlsx
+++ b/12-upload_file_merge_file/output/pub_cd_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\12-upload_file_merge_file\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87441041-F18D-4D5F-8A53-F8EAAF4E43FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC0EA77C-5541-4336-B7D3-491BEC3184AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="23452" windowHeight="12561" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="375" yWindow="375" windowWidth="17425" windowHeight="8955" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rem-代码映射" sheetId="1" r:id="rId1"/>
@@ -25,122 +25,123 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+  <si>
+    <t>SRC_TAB_LIB_NAME</t>
+  </si>
+  <si>
+    <t>SRC_TAB_EN_NAME</t>
+  </si>
+  <si>
+    <t>SRC_TAB_CN_NAME</t>
+  </si>
+  <si>
+    <t>SRC_FIELD_EN_NAME</t>
+  </si>
+  <si>
+    <t>SRC_FIELD_CN_NAME</t>
+  </si>
+  <si>
+    <t>SRC_CD_VAL</t>
+  </si>
+  <si>
+    <t>SRC_CD_DESC</t>
+  </si>
+  <si>
+    <t>TARGRT_TAB_EN_NAME</t>
+  </si>
+  <si>
+    <t>TARGRT_TAB_CN_NAME</t>
+  </si>
+  <si>
+    <t>TARGRT_FIELD_EN_NAME</t>
+  </si>
+  <si>
+    <t>TARGRT_FIELD_CN_NAME</t>
+  </si>
+  <si>
+    <t>TARGET_CD_VAL</t>
+  </si>
+  <si>
+    <t>TARGET_CD_DESC</t>
+  </si>
+  <si>
+    <t>REM</t>
+  </si>
   <si>
     <t>取数来源应用</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>取数来源表中文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>取数来源表英文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>取数来源字段中文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>取数来源字段英文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>源代码码值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>源代码码值说明</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标表中文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标表英文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标字段中文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标字段英文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标代码码值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>目标代码说明</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>特殊说明</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>REM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGET_CD_DESC</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGET_CD_VAL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGRT_FIELD_CN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGRT_FIELD_EN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGRT_TAB_CN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TARGRT_TAB_EN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_CD_DESC</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_CD_VAL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_FIELD_CN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_FIELD_EN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_TAB_CN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_TAB_EN_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SRC_TAB_LIB_NAME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>line4444444</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LINE1111111</t>
+  </si>
+  <si>
+    <t>line1111111</t>
+  </si>
+  <si>
+    <t>line2222222</t>
+  </si>
+  <si>
+    <t>LINE2222222</t>
+  </si>
+  <si>
+    <t>line3333333</t>
+  </si>
+  <si>
+    <t>LINE3333333</t>
+  </si>
+  <si>
+    <t>line55555</t>
+  </si>
+  <si>
+    <t>LINE55555</t>
+  </si>
+  <si>
+    <t>line66666</t>
+  </si>
+  <si>
+    <t>LINE66666</t>
   </si>
 </sst>
 </file>
@@ -499,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="13.95" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.5546875" customWidth="1"/>
@@ -509,90 +510,90 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="22.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -680,6 +681,622 @@
         <v>2</v>
       </c>
       <c r="N4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+      <c r="N5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+      <c r="N6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>2</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7">
+        <v>2</v>
+      </c>
+      <c r="N7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8">
+        <v>2</v>
+      </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>31</v>
+      </c>
+      <c r="I9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9">
+        <v>2</v>
+      </c>
+      <c r="K9">
+        <v>2</v>
+      </c>
+      <c r="L9">
+        <v>2</v>
+      </c>
+      <c r="M9">
+        <v>2</v>
+      </c>
+      <c r="N9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" t="s">
+        <v>32</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10">
+        <v>2</v>
+      </c>
+      <c r="N10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <v>2</v>
+      </c>
+      <c r="M11">
+        <v>2</v>
+      </c>
+      <c r="N11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J12">
+        <v>2</v>
+      </c>
+      <c r="K12">
+        <v>2</v>
+      </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
+      <c r="M12">
+        <v>2</v>
+      </c>
+      <c r="N12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J13">
+        <v>2</v>
+      </c>
+      <c r="K13">
+        <v>2</v>
+      </c>
+      <c r="L13">
+        <v>2</v>
+      </c>
+      <c r="M13">
+        <v>2</v>
+      </c>
+      <c r="N13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" t="s">
+        <v>36</v>
+      </c>
+      <c r="J14">
+        <v>2</v>
+      </c>
+      <c r="K14">
+        <v>2</v>
+      </c>
+      <c r="L14">
+        <v>2</v>
+      </c>
+      <c r="M14">
+        <v>2</v>
+      </c>
+      <c r="N14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15">
+        <v>2</v>
+      </c>
+      <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="L15">
+        <v>2</v>
+      </c>
+      <c r="M15">
+        <v>2</v>
+      </c>
+      <c r="N15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" t="s">
+        <v>36</v>
+      </c>
+      <c r="J16">
+        <v>2</v>
+      </c>
+      <c r="K16">
+        <v>2</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16">
+        <v>2</v>
+      </c>
+      <c r="N16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I17" t="s">
+        <v>38</v>
+      </c>
+      <c r="J17">
+        <v>2</v>
+      </c>
+      <c r="K17">
+        <v>2</v>
+      </c>
+      <c r="L17">
+        <v>2</v>
+      </c>
+      <c r="M17">
+        <v>2</v>
+      </c>
+      <c r="N17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" t="s">
+        <v>38</v>
+      </c>
+      <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
+      <c r="L18">
+        <v>2</v>
+      </c>
+      <c r="M18">
+        <v>2</v>
+      </c>
+      <c r="N18">
         <v>2</v>
       </c>
     </row>

</xml_diff>